<commit_message>
feat: adiciona semana atual automática na saudação e no formulário
* Implementa função para cálculo da semana do ano (ISO 8601)
* Exibe a semana atual junto com a data na saudação
* Preenche automaticamente o campo Week ao carregar a página
* Garante sincronização entre saudação e formulário
* Ajusta reset do formulário para manter semana atual
</commit_message>
<xml_diff>
--- a/data/relatorios.xlsx
+++ b/data/relatorios.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L861"/>
+  <dimension ref="A1:L935"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7081,7 +7081,7 @@
         <v>ANÁLISE DIMENSIONAL</v>
       </c>
       <c r="K176" t="str" xml:space="preserve">
-        <v xml:space="preserve">PREVENTIVA_x000d__x000d__x000d_
+        <v xml:space="preserve">PREVENTIVA_x000d__x000d__x000d__x000d__x000d_
 </v>
       </c>
       <c r="L176" t="b">
@@ -7804,7 +7804,7 @@
         <v>ANÁLISE DIMENSIONAL</v>
       </c>
       <c r="K195" t="str" xml:space="preserve">
-        <v xml:space="preserve">PEÇA 02 DA BASE A1_x000d__x000d__x000d_
+        <v xml:space="preserve">PEÇA 02 DA BASE A1_x000d__x000d__x000d__x000d__x000d_
 </v>
       </c>
       <c r="L195" t="b">
@@ -13885,7 +13885,7 @@
         <v>ANÁLISE DIMENSIONAL</v>
       </c>
       <c r="K355" t="str" xml:space="preserve">
-        <v xml:space="preserve">PEÇAS EM DESVIO_x000d__x000d__x000d_
+        <v xml:space="preserve">PEÇAS EM DESVIO_x000d__x000d__x000d__x000d__x000d_
 </v>
       </c>
       <c r="L355" t="b">
@@ -13924,7 +13924,7 @@
         <v>ANÁLISE DIMENSIONAL</v>
       </c>
       <c r="K356" t="str" xml:space="preserve">
-        <v xml:space="preserve">PEÇAS EM DESVIO_x000d__x000d__x000d_
+        <v xml:space="preserve">PEÇAS EM DESVIO_x000d__x000d__x000d__x000d__x000d_
 </v>
       </c>
       <c r="L356" t="b">
@@ -23083,7 +23083,7 @@
         <v>ANÁLISE DIMENSIONAL</v>
       </c>
       <c r="K597" t="str" xml:space="preserve">
-        <v xml:space="preserve">PRODUÇÃO APÓS ATUAÇÃO DA FERRAMENTARIA_x000d__x000d__x000d_
+        <v xml:space="preserve">PRODUÇÃO APÓS ATUAÇÃO DA FERRAMENTARIA_x000d__x000d__x000d__x000d__x000d_
 </v>
       </c>
       <c r="L597" t="b">
@@ -23122,7 +23122,7 @@
         <v>ANÁLISE DIMENSIONAL</v>
       </c>
       <c r="K598" t="str" xml:space="preserve">
-        <v xml:space="preserve">PRODUÇÃO APÓS ATUAÇÃO DA FERRAMENTARIA_x000d__x000d__x000d_
+        <v xml:space="preserve">PRODUÇÃO APÓS ATUAÇÃO DA FERRAMENTARIA_x000d__x000d__x000d__x000d__x000d_
 </v>
       </c>
       <c r="L598" t="b">
@@ -33123,9 +33123,2821 @@
         <v>0</v>
       </c>
     </row>
+    <row r="862">
+      <c r="A862" t="str">
+        <v>C2026.0861</v>
+      </c>
+      <c r="B862" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C862" t="str">
+        <v>53377061</v>
+      </c>
+      <c r="D862" t="str">
+        <v>PRISMA</v>
+      </c>
+      <c r="E862" t="str">
+        <v>15</v>
+      </c>
+      <c r="F862" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G862" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H862" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I862" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J862" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K862" t="str">
+        <v/>
+      </c>
+      <c r="L862" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="str">
+        <v>C2026.0862</v>
+      </c>
+      <c r="B863" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C863" t="str">
+        <v>53377061</v>
+      </c>
+      <c r="D863" t="str">
+        <v>PRISMA</v>
+      </c>
+      <c r="E863" t="str">
+        <v>15</v>
+      </c>
+      <c r="F863" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G863" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H863" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I863" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J863" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K863" t="str">
+        <v/>
+      </c>
+      <c r="L863" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="str">
+        <v>C2026.0863</v>
+      </c>
+      <c r="B864" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C864" t="str">
+        <v>53497979</v>
+      </c>
+      <c r="D864" t="str">
+        <v>SCONTRINO SERRATURA COFANO</v>
+      </c>
+      <c r="E864" t="str">
+        <v>15</v>
+      </c>
+      <c r="F864" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G864" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H864" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I864" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J864" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K864" t="str">
+        <v/>
+      </c>
+      <c r="L864" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="str">
+        <v>C2026.0864</v>
+      </c>
+      <c r="B865" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C865" t="str">
+        <v>521432780</v>
+      </c>
+      <c r="D865" t="str">
+        <v>SERRATURA COFANO</v>
+      </c>
+      <c r="E865" t="str">
+        <v>15</v>
+      </c>
+      <c r="F865" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G865" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H865" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I865" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J865" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K865" t="str">
+        <v/>
+      </c>
+      <c r="L865" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="str">
+        <v>C2026.0865</v>
+      </c>
+      <c r="B866" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C866" t="str">
+        <v>53497979</v>
+      </c>
+      <c r="D866" t="str">
+        <v>SCONTRINO SERRATURA COFANO</v>
+      </c>
+      <c r="E866" t="str">
+        <v>15</v>
+      </c>
+      <c r="F866" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G866" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H866" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I866" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J866" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K866" t="str">
+        <v/>
+      </c>
+      <c r="L866" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="str">
+        <v>C2026.0866</v>
+      </c>
+      <c r="B867" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C867" t="str">
+        <v>53497979</v>
+      </c>
+      <c r="D867" t="str">
+        <v>SCONTRINO SERRATURA COFANO</v>
+      </c>
+      <c r="E867" t="str">
+        <v>15</v>
+      </c>
+      <c r="F867" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G867" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H867" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I867" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J867" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K867" t="str">
+        <v/>
+      </c>
+      <c r="L867" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="str">
+        <v>C2026.0867</v>
+      </c>
+      <c r="B868" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C868" t="str">
+        <v>53497979</v>
+      </c>
+      <c r="D868" t="str">
+        <v>SCONTRINO SERRATURA COFANO</v>
+      </c>
+      <c r="E868" t="str">
+        <v>15</v>
+      </c>
+      <c r="F868" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G868" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H868" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I868" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J868" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K868" t="str">
+        <v/>
+      </c>
+      <c r="L868" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="str">
+        <v>C2026.0868</v>
+      </c>
+      <c r="B869" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C869" t="str">
+        <v>53497979</v>
+      </c>
+      <c r="D869" t="str">
+        <v>SCONTRINO SERRATURA COFANO</v>
+      </c>
+      <c r="E869" t="str">
+        <v>15</v>
+      </c>
+      <c r="F869" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G869" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H869" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I869" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J869" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K869" t="str">
+        <v/>
+      </c>
+      <c r="L869" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="str">
+        <v>C2026.0869</v>
+      </c>
+      <c r="B870" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C870" t="str">
+        <v>53498105</v>
+      </c>
+      <c r="D870" t="str">
+        <v>CUCÃO DX</v>
+      </c>
+      <c r="E870" t="str">
+        <v>15</v>
+      </c>
+      <c r="F870" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G870" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H870" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I870" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J870" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K870" t="str">
+        <v/>
+      </c>
+      <c r="L870" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="str">
+        <v>C2026.0870</v>
+      </c>
+      <c r="B871" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C871" t="str">
+        <v>53498106</v>
+      </c>
+      <c r="D871" t="str">
+        <v>CUCÃO SX</v>
+      </c>
+      <c r="E871" t="str">
+        <v>15</v>
+      </c>
+      <c r="F871" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G871" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H871" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I871" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J871" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K871" t="str">
+        <v/>
+      </c>
+      <c r="L871" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="str">
+        <v>C2026.0871</v>
+      </c>
+      <c r="B872" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C872" t="str">
+        <v>52143278</v>
+      </c>
+      <c r="D872" t="str">
+        <v>SERRATURA COFANO CPL</v>
+      </c>
+      <c r="E872" t="str">
+        <v>15</v>
+      </c>
+      <c r="F872" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G872" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H872" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I872" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J872" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K872" t="str">
+        <v/>
+      </c>
+      <c r="L872" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="str">
+        <v>C2026.0872</v>
+      </c>
+      <c r="B873" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C873" t="str">
+        <v>52143278</v>
+      </c>
+      <c r="D873" t="str">
+        <v>SERRATURA COFANO CPL</v>
+      </c>
+      <c r="E873" t="str">
+        <v>15</v>
+      </c>
+      <c r="F873" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G873" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H873" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I873" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J873" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K873" t="str">
+        <v/>
+      </c>
+      <c r="L873" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="str">
+        <v>C2026.0873</v>
+      </c>
+      <c r="B874" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C874" t="str">
+        <v>52143278</v>
+      </c>
+      <c r="D874" t="str">
+        <v>SERRATURA COFANO CPL</v>
+      </c>
+      <c r="E874" t="str">
+        <v>15</v>
+      </c>
+      <c r="F874" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G874" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H874" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I874" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J874" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K874" t="str">
+        <v/>
+      </c>
+      <c r="L874" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="str">
+        <v>C2026.0874</v>
+      </c>
+      <c r="B875" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C875" t="str">
+        <v>52143278</v>
+      </c>
+      <c r="D875" t="str">
+        <v>SERRATURA COFANO CPL</v>
+      </c>
+      <c r="E875" t="str">
+        <v>15</v>
+      </c>
+      <c r="F875" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G875" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H875" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I875" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J875" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K875" t="str">
+        <v/>
+      </c>
+      <c r="L875" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="str">
+        <v>C2026.0875</v>
+      </c>
+      <c r="B876" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C876" t="str">
+        <v>52143278</v>
+      </c>
+      <c r="D876" t="str">
+        <v>SERRATURA COFANO CPL</v>
+      </c>
+      <c r="E876" t="str">
+        <v>15</v>
+      </c>
+      <c r="F876" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G876" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H876" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I876" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J876" t="str">
+        <v>PPAP</v>
+      </c>
+      <c r="K876" t="str">
+        <v/>
+      </c>
+      <c r="L876" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="str">
+        <v>C2026.0876</v>
+      </c>
+      <c r="B877" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C877" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D877" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E877" t="str">
+        <v>15</v>
+      </c>
+      <c r="F877" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G877" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H877" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I877" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J877" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K877" t="str">
+        <v/>
+      </c>
+      <c r="L877" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="str">
+        <v>C2026.0877</v>
+      </c>
+      <c r="B878" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C878" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D878" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E878" t="str">
+        <v>15</v>
+      </c>
+      <c r="F878" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G878" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H878" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I878" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J878" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K878" t="str">
+        <v/>
+      </c>
+      <c r="L878" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="str">
+        <v>C2026.0878</v>
+      </c>
+      <c r="B879" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C879" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D879" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E879" t="str">
+        <v>15</v>
+      </c>
+      <c r="F879" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G879" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H879" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I879" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J879" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K879" t="str">
+        <v/>
+      </c>
+      <c r="L879" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="str">
+        <v>C2026.0879</v>
+      </c>
+      <c r="B880" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C880" t="str">
+        <v>51966401</v>
+      </c>
+      <c r="D880" t="str">
+        <v>SIDE BAR SUPPORTO DI SCORTA</v>
+      </c>
+      <c r="E880" t="str">
+        <v>15</v>
+      </c>
+      <c r="F880" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G880" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H880" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I880" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J880" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K880" t="str">
+        <v>PRODUÇÃO 06/04/2026</v>
+      </c>
+      <c r="L880" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="str">
+        <v>C2026.0880</v>
+      </c>
+      <c r="B881" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C881" t="str">
+        <v>51966402</v>
+      </c>
+      <c r="D881" t="str">
+        <v>SIDE BAR SUPPORTO DI SCORTA</v>
+      </c>
+      <c r="E881" t="str">
+        <v>15</v>
+      </c>
+      <c r="F881" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G881" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H881" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I881" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J881" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K881" t="str">
+        <v>PRODUÇÃO 06/04/2027</v>
+      </c>
+      <c r="L881" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="str">
+        <v>C2026.0881</v>
+      </c>
+      <c r="B882" t="str">
+        <v>06/04/2026</v>
+      </c>
+      <c r="C882" t="str">
+        <v>51966400</v>
+      </c>
+      <c r="D882" t="str">
+        <v>BRACKET CENTRAL CS</v>
+      </c>
+      <c r="E882" t="str">
+        <v>15</v>
+      </c>
+      <c r="F882" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G882" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H882" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I882" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J882" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K882" t="str">
+        <v/>
+      </c>
+      <c r="L882" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="str">
+        <v>C2026.0882</v>
+      </c>
+      <c r="B883" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C883" t="str">
+        <v>53416452</v>
+      </c>
+      <c r="D883" t="str">
+        <v>CUCÃO DX</v>
+      </c>
+      <c r="E883" t="str">
+        <v>15</v>
+      </c>
+      <c r="F883" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G883" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H883" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I883" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J883" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K883" t="str">
+        <v/>
+      </c>
+      <c r="L883" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="str">
+        <v>C2026.0883</v>
+      </c>
+      <c r="B884" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C884" t="str">
+        <v>53416453</v>
+      </c>
+      <c r="D884" t="str">
+        <v>CUCÃO SX</v>
+      </c>
+      <c r="E884" t="str">
+        <v>15</v>
+      </c>
+      <c r="F884" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G884" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H884" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I884" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J884" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K884" t="str">
+        <v/>
+      </c>
+      <c r="L884" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="str">
+        <v>C2026.0884</v>
+      </c>
+      <c r="B885" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C885" t="str">
+        <v>53490364</v>
+      </c>
+      <c r="D885" t="str">
+        <v>BRACKET COMPL. SX</v>
+      </c>
+      <c r="E885" t="str">
+        <v>15</v>
+      </c>
+      <c r="F885" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G885" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H885" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I885" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J885" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K885" t="str">
+        <v/>
+      </c>
+      <c r="L885" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="str">
+        <v>C2026.0885</v>
+      </c>
+      <c r="B886" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C886" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D886" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E886" t="str">
+        <v>15</v>
+      </c>
+      <c r="F886" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G886" t="str">
+        <v>izaac</v>
+      </c>
+      <c r="H886" t="str">
+        <v>ADM</v>
+      </c>
+      <c r="I886" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J886" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K886" t="str">
+        <v/>
+      </c>
+      <c r="L886" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="str">
+        <v>C2026.0886</v>
+      </c>
+      <c r="B887" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C887" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D887" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E887" t="str">
+        <v>15</v>
+      </c>
+      <c r="F887" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G887" t="str">
+        <v>izaac</v>
+      </c>
+      <c r="H887" t="str">
+        <v>ADM</v>
+      </c>
+      <c r="I887" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J887" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K887" t="str">
+        <v/>
+      </c>
+      <c r="L887" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="str">
+        <v>C2026.0887</v>
+      </c>
+      <c r="B888" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C888" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D888" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E888" t="str">
+        <v>15</v>
+      </c>
+      <c r="F888" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G888" t="str">
+        <v>izaac</v>
+      </c>
+      <c r="H888" t="str">
+        <v>ADM</v>
+      </c>
+      <c r="I888" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J888" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K888" t="str">
+        <v/>
+      </c>
+      <c r="L888" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="str">
+        <v>C2026.0888</v>
+      </c>
+      <c r="B889" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C889" t="str">
+        <v>53490309</v>
+      </c>
+      <c r="D889" t="str">
+        <v>BRACKET COMPL. DX</v>
+      </c>
+      <c r="E889" t="str">
+        <v>15</v>
+      </c>
+      <c r="F889" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G889" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H889" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I889" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J889" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K889" t="str">
+        <v/>
+      </c>
+      <c r="L889" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="str">
+        <v>C2026.0889</v>
+      </c>
+      <c r="B890" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C890" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D890" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E890" t="str">
+        <v>15</v>
+      </c>
+      <c r="F890" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G890" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H890" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I890" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J890" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K890" t="str">
+        <v/>
+      </c>
+      <c r="L890" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="str">
+        <v>C2026.0890</v>
+      </c>
+      <c r="B891" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C891" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D891" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E891" t="str">
+        <v>15</v>
+      </c>
+      <c r="F891" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G891" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H891" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I891" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J891" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K891" t="str">
+        <v/>
+      </c>
+      <c r="L891" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="str">
+        <v>C2026.0891</v>
+      </c>
+      <c r="B892" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C892" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D892" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E892" t="str">
+        <v>15</v>
+      </c>
+      <c r="F892" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G892" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H892" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I892" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J892" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K892" t="str">
+        <v/>
+      </c>
+      <c r="L892" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="str">
+        <v>C2026.0892</v>
+      </c>
+      <c r="B893" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C893" t="str">
+        <v>53328140</v>
+      </c>
+      <c r="D893" t="str">
+        <v>RACKET ASSY F. M. FRT LT</v>
+      </c>
+      <c r="E893" t="str">
+        <v>15</v>
+      </c>
+      <c r="F893" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G893" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H893" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I893" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J893" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K893" t="str">
+        <v/>
+      </c>
+      <c r="L893" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="str">
+        <v>C2026.0893</v>
+      </c>
+      <c r="B894" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C894" t="str">
+        <v>53328139</v>
+      </c>
+      <c r="D894" t="str">
+        <v>BRACKET ASSY FENDER MOUNTING FRT RT</v>
+      </c>
+      <c r="E894" t="str">
+        <v>15</v>
+      </c>
+      <c r="F894" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G894" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H894" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I894" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J894" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K894" t="str">
+        <v/>
+      </c>
+      <c r="L894" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="str">
+        <v>C2026.0894</v>
+      </c>
+      <c r="B895" t="str">
+        <v>07/04/2026</v>
+      </c>
+      <c r="C895" t="str">
+        <v>53489451</v>
+      </c>
+      <c r="D895" t="str">
+        <v>SIDE SILL SX</v>
+      </c>
+      <c r="E895" t="str">
+        <v>15</v>
+      </c>
+      <c r="F895" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G895" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H895" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I895" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J895" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K895" t="str">
+        <v/>
+      </c>
+      <c r="L895" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="str">
+        <v>C2026.0895</v>
+      </c>
+      <c r="B896" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C896" t="str">
+        <v>53327241</v>
+      </c>
+      <c r="D896" t="str">
+        <v>MÃO FRANCESA</v>
+      </c>
+      <c r="E896" t="str">
+        <v>15</v>
+      </c>
+      <c r="F896" t="str">
+        <v>ENGENHARIA</v>
+      </c>
+      <c r="G896" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H896" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I896" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J896" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K896" t="str">
+        <v/>
+      </c>
+      <c r="L896" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="str">
+        <v>C2026.0896</v>
+      </c>
+      <c r="B897" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C897" t="str">
+        <v>53328139</v>
+      </c>
+      <c r="D897" t="str">
+        <v>TORRESMO DX</v>
+      </c>
+      <c r="E897" t="str">
+        <v>15</v>
+      </c>
+      <c r="F897" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G897" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H897" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I897" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J897" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K897" t="str">
+        <v/>
+      </c>
+      <c r="L897" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="str">
+        <v>C2026.0897</v>
+      </c>
+      <c r="B898" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C898" t="str">
+        <v>53327786</v>
+      </c>
+      <c r="D898" t="str">
+        <v>bendita dx</v>
+      </c>
+      <c r="E898" t="str">
+        <v>15</v>
+      </c>
+      <c r="F898" t="str">
+        <v>FERRAMENTARIA</v>
+      </c>
+      <c r="G898" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H898" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I898" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J898" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K898" t="str">
+        <v/>
+      </c>
+      <c r="L898" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="str">
+        <v>C2026.0898</v>
+      </c>
+      <c r="B899" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C899" t="str">
+        <v>53327797</v>
+      </c>
+      <c r="D899" t="str">
+        <v>BENDITA SX</v>
+      </c>
+      <c r="E899" t="str">
+        <v>15</v>
+      </c>
+      <c r="F899" t="str">
+        <v>FERRAMENTARIA</v>
+      </c>
+      <c r="G899" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H899" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I899" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J899" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K899" t="str">
+        <v/>
+      </c>
+      <c r="L899" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="str">
+        <v>C2026.0899</v>
+      </c>
+      <c r="B900" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C900" t="str">
+        <v>53328140</v>
+      </c>
+      <c r="D900" t="str">
+        <v>TORRESMO SX</v>
+      </c>
+      <c r="E900" t="str">
+        <v>15</v>
+      </c>
+      <c r="F900" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G900" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H900" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I900" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J900" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K900" t="str">
+        <v/>
+      </c>
+      <c r="L900" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="str">
+        <v>C2026.0900</v>
+      </c>
+      <c r="B901" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C901" t="str">
+        <v>53377061</v>
+      </c>
+      <c r="D901" t="str">
+        <v>PRISMA</v>
+      </c>
+      <c r="E901" t="str">
+        <v>15</v>
+      </c>
+      <c r="F901" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G901" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H901" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I901" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J901" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K901" t="str">
+        <v/>
+      </c>
+      <c r="L901" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="str">
+        <v>C2026.0901</v>
+      </c>
+      <c r="B902" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C902" t="str">
+        <v>53377061</v>
+      </c>
+      <c r="D902" t="str">
+        <v>RINFORZO SERRATURA PORTELLONE</v>
+      </c>
+      <c r="E902" t="str">
+        <v>15</v>
+      </c>
+      <c r="F902" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G902" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H902" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I902" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J902" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K902" t="str">
+        <v/>
+      </c>
+      <c r="L902" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="str">
+        <v>C2026.0902</v>
+      </c>
+      <c r="B903" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C903" t="str">
+        <v>53327797</v>
+      </c>
+      <c r="D903" t="str">
+        <v>SUPPORTO CS. MODULO FRONT END SX</v>
+      </c>
+      <c r="E903" t="str">
+        <v>15</v>
+      </c>
+      <c r="F903" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G903" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H903" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I903" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J903" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K903" t="str">
+        <v/>
+      </c>
+      <c r="L903" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="str">
+        <v>C2026.0903</v>
+      </c>
+      <c r="B904" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C904" t="str">
+        <v>53327786</v>
+      </c>
+      <c r="D904" t="str">
+        <v>SUPPORTO CS. MODULO FRONT END DX</v>
+      </c>
+      <c r="E904" t="str">
+        <v>15</v>
+      </c>
+      <c r="F904" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G904" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H904" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I904" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J904" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K904" t="str">
+        <v/>
+      </c>
+      <c r="L904" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="str">
+        <v>C2026.0904</v>
+      </c>
+      <c r="B905" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C905" t="str">
+        <v>53327786</v>
+      </c>
+      <c r="D905" t="str">
+        <v>SUPPORTO CS. MODULO FRONT END DX</v>
+      </c>
+      <c r="E905" t="str">
+        <v>15</v>
+      </c>
+      <c r="F905" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G905" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H905" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I905" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J905" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K905" t="str">
+        <v/>
+      </c>
+      <c r="L905" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="str">
+        <v>C2026.0905</v>
+      </c>
+      <c r="B906" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C906" t="str">
+        <v>53489448</v>
+      </c>
+      <c r="D906" t="str">
+        <v>SIDE SILL DX</v>
+      </c>
+      <c r="E906" t="str">
+        <v>15</v>
+      </c>
+      <c r="F906" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G906" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H906" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I906" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J906" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K906" t="str">
+        <v/>
+      </c>
+      <c r="L906" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="str">
+        <v>C2026.0906</v>
+      </c>
+      <c r="B907" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C907" t="str">
+        <v>53489448</v>
+      </c>
+      <c r="D907" t="str">
+        <v>SIDE SILL DX</v>
+      </c>
+      <c r="E907" t="str">
+        <v>15</v>
+      </c>
+      <c r="F907" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G907" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H907" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I907" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J907" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K907" t="str">
+        <v/>
+      </c>
+      <c r="L907" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="str">
+        <v>C2026.0907</v>
+      </c>
+      <c r="B908" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C908" t="str">
+        <v>53489448</v>
+      </c>
+      <c r="D908" t="str">
+        <v>SIDE SILL DX</v>
+      </c>
+      <c r="E908" t="str">
+        <v>15</v>
+      </c>
+      <c r="F908" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G908" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H908" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I908" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J908" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K908" t="str">
+        <v/>
+      </c>
+      <c r="L908" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="str">
+        <v>C2026.0908</v>
+      </c>
+      <c r="B909" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C909" t="str">
+        <v>53489448</v>
+      </c>
+      <c r="D909" t="str">
+        <v>SIDE SILL DX</v>
+      </c>
+      <c r="E909" t="str">
+        <v>15</v>
+      </c>
+      <c r="F909" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G909" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H909" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I909" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J909" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K909" t="str">
+        <v/>
+      </c>
+      <c r="L909" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="str">
+        <v>C2026.0909</v>
+      </c>
+      <c r="B910" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C910" t="str">
+        <v>53489448</v>
+      </c>
+      <c r="D910" t="str">
+        <v>SIDE SILL DX</v>
+      </c>
+      <c r="E910" t="str">
+        <v>15</v>
+      </c>
+      <c r="F910" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G910" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H910" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I910" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J910" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K910" t="str">
+        <v/>
+      </c>
+      <c r="L910" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="str">
+        <v>C2026.0910</v>
+      </c>
+      <c r="B911" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C911" t="str">
+        <v>53327793</v>
+      </c>
+      <c r="D911" t="str">
+        <v>REINF. BULKHEAD SX</v>
+      </c>
+      <c r="E911" t="str">
+        <v>15</v>
+      </c>
+      <c r="F911" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G911" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H911" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I911" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J911" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K911" t="str">
+        <v/>
+      </c>
+      <c r="L911" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="str">
+        <v>C2026.0911</v>
+      </c>
+      <c r="B912" t="str">
+        <v>08/04/2026</v>
+      </c>
+      <c r="C912" t="str">
+        <v>53327782</v>
+      </c>
+      <c r="D912" t="str">
+        <v>REINF. BULKHEAD DX</v>
+      </c>
+      <c r="E912" t="str">
+        <v>15</v>
+      </c>
+      <c r="F912" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G912" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H912" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I912" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J912" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K912" t="str">
+        <v/>
+      </c>
+      <c r="L912" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="str">
+        <v>C2026.0912</v>
+      </c>
+      <c r="B913" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C913" t="str">
+        <v>52225420</v>
+      </c>
+      <c r="D913" t="str">
+        <v>PONTEIRA SX</v>
+      </c>
+      <c r="E913" t="str">
+        <v>15</v>
+      </c>
+      <c r="F913" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G913" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H913" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I913" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J913" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K913" t="str">
+        <v/>
+      </c>
+      <c r="L913" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="str">
+        <v>C2026.0913</v>
+      </c>
+      <c r="B914" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C914" t="str">
+        <v>53376480</v>
+      </c>
+      <c r="D914" t="str">
+        <v>PONTEIRA DX</v>
+      </c>
+      <c r="E914" t="str">
+        <v>15</v>
+      </c>
+      <c r="F914" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G914" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H914" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I914" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J914" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K914" t="str">
+        <v/>
+      </c>
+      <c r="L914" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="str">
+        <v>C2026.0914</v>
+      </c>
+      <c r="B915" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C915" t="str">
+        <v>53489530</v>
+      </c>
+      <c r="D915" t="str">
+        <v>CALÇO 03 DX</v>
+      </c>
+      <c r="E915" t="str">
+        <v>15</v>
+      </c>
+      <c r="F915" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G915" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H915" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I915" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J915" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K915" t="str">
+        <v/>
+      </c>
+      <c r="L915" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="str">
+        <v>C2026.0915</v>
+      </c>
+      <c r="B916" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C916" t="str">
+        <v>53489530</v>
+      </c>
+      <c r="D916" t="str">
+        <v>CALÇO 03 DX</v>
+      </c>
+      <c r="E916" t="str">
+        <v>15</v>
+      </c>
+      <c r="F916" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G916" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H916" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I916" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J916" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K916" t="str">
+        <v/>
+      </c>
+      <c r="L916" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="str">
+        <v>C2026.0916</v>
+      </c>
+      <c r="B917" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C917" t="str">
+        <v>53489530</v>
+      </c>
+      <c r="D917" t="str">
+        <v>CALÇO 03 DX</v>
+      </c>
+      <c r="E917" t="str">
+        <v>15</v>
+      </c>
+      <c r="F917" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G917" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H917" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I917" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J917" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K917" t="str">
+        <v/>
+      </c>
+      <c r="L917" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="str">
+        <v>C2026.0917</v>
+      </c>
+      <c r="B918" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C918" t="str">
+        <v>53489530</v>
+      </c>
+      <c r="D918" t="str">
+        <v>CALÇO 03 DX</v>
+      </c>
+      <c r="E918" t="str">
+        <v>15</v>
+      </c>
+      <c r="F918" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G918" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H918" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I918" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J918" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K918" t="str">
+        <v/>
+      </c>
+      <c r="L918" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="str">
+        <v>C2026.0918</v>
+      </c>
+      <c r="B919" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C919" t="str">
+        <v>53490336</v>
+      </c>
+      <c r="D919" t="str">
+        <v>CALÇO 01 DX</v>
+      </c>
+      <c r="E919" t="str">
+        <v>15</v>
+      </c>
+      <c r="F919" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G919" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H919" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I919" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J919" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K919" t="str">
+        <v/>
+      </c>
+      <c r="L919" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="str">
+        <v>C2026.0919</v>
+      </c>
+      <c r="B920" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C920" t="str">
+        <v>53490336</v>
+      </c>
+      <c r="D920" t="str">
+        <v>CALÇO 01 DX</v>
+      </c>
+      <c r="E920" t="str">
+        <v>15</v>
+      </c>
+      <c r="F920" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G920" t="str">
+        <v>matheus</v>
+      </c>
+      <c r="H920" t="str">
+        <v>1º TURNO</v>
+      </c>
+      <c r="I920" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J920" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K920" t="str">
+        <v/>
+      </c>
+      <c r="L920" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="str">
+        <v>C2026.0920</v>
+      </c>
+      <c r="B921" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C921" t="str">
+        <v>53359033</v>
+      </c>
+      <c r="D921" t="str">
+        <v>BRACKET RR FASCIA ATTACK SING</v>
+      </c>
+      <c r="E921" t="str">
+        <v>15</v>
+      </c>
+      <c r="F921" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G921" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H921" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I921" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J921" t="str">
+        <v>INSP LAYOUT</v>
+      </c>
+      <c r="K921" t="str">
+        <v/>
+      </c>
+      <c r="L921" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="str">
+        <v>C2026.0921</v>
+      </c>
+      <c r="B922" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C922" t="str">
+        <v>53359033</v>
+      </c>
+      <c r="D922" t="str">
+        <v>BRACKET RR FASCIA ATTACK SING</v>
+      </c>
+      <c r="E922" t="str">
+        <v>15</v>
+      </c>
+      <c r="F922" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G922" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H922" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I922" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J922" t="str">
+        <v>INSP LAYOUT</v>
+      </c>
+      <c r="K922" t="str">
+        <v/>
+      </c>
+      <c r="L922" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="str">
+        <v>C2026.0922</v>
+      </c>
+      <c r="B923" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C923" t="str">
+        <v>53359033</v>
+      </c>
+      <c r="D923" t="str">
+        <v>BRACKET RR FASCIA ATTACK SING</v>
+      </c>
+      <c r="E923" t="str">
+        <v>15</v>
+      </c>
+      <c r="F923" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G923" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H923" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I923" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J923" t="str">
+        <v>INSP LAYOUT</v>
+      </c>
+      <c r="K923" t="str">
+        <v/>
+      </c>
+      <c r="L923" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="str">
+        <v>C2026.0923</v>
+      </c>
+      <c r="B924" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C924" t="str">
+        <v>53359033</v>
+      </c>
+      <c r="D924" t="str">
+        <v>BRACKET RR FASCIA ATTACK SING</v>
+      </c>
+      <c r="E924" t="str">
+        <v>15</v>
+      </c>
+      <c r="F924" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G924" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H924" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I924" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J924" t="str">
+        <v>INSP LAYOUT</v>
+      </c>
+      <c r="K924" t="str">
+        <v/>
+      </c>
+      <c r="L924" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="str">
+        <v>C2026.0924</v>
+      </c>
+      <c r="B925" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C925" t="str">
+        <v>53359033</v>
+      </c>
+      <c r="D925" t="str">
+        <v>BRACKET RR FASCIA ATTACK SING</v>
+      </c>
+      <c r="E925" t="str">
+        <v>15</v>
+      </c>
+      <c r="F925" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G925" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H925" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I925" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J925" t="str">
+        <v>INSP LAYOUT</v>
+      </c>
+      <c r="K925" t="str">
+        <v/>
+      </c>
+      <c r="L925" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="str">
+        <v>C2026.0925</v>
+      </c>
+      <c r="B926" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C926" t="str">
+        <v>53489671</v>
+      </c>
+      <c r="D926" t="str">
+        <v>CONJUNTO TRANSVERSAL TRASEIRO</v>
+      </c>
+      <c r="E926" t="str">
+        <v>15</v>
+      </c>
+      <c r="F926" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G926" t="str">
+        <v>izaac</v>
+      </c>
+      <c r="H926" t="str">
+        <v>ADM</v>
+      </c>
+      <c r="I926" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J926" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K926" t="str">
+        <v/>
+      </c>
+      <c r="L926" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="str">
+        <v>C2026.0926</v>
+      </c>
+      <c r="B927" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C927" t="str">
+        <v>53489671</v>
+      </c>
+      <c r="D927" t="str">
+        <v>CONJUNTO TRANSVERSAL TRASEIRO</v>
+      </c>
+      <c r="E927" t="str">
+        <v>15</v>
+      </c>
+      <c r="F927" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G927" t="str">
+        <v>izaac</v>
+      </c>
+      <c r="H927" t="str">
+        <v>ADM</v>
+      </c>
+      <c r="I927" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J927" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K927" t="str">
+        <v/>
+      </c>
+      <c r="L927" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="str">
+        <v>C2026.0927</v>
+      </c>
+      <c r="B928" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C928" t="str">
+        <v>53489671</v>
+      </c>
+      <c r="D928" t="str">
+        <v>CONJUNTO TRANSVERSAL TRASEIRO</v>
+      </c>
+      <c r="E928" t="str">
+        <v>15</v>
+      </c>
+      <c r="F928" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G928" t="str">
+        <v>izaac</v>
+      </c>
+      <c r="H928" t="str">
+        <v>ADM</v>
+      </c>
+      <c r="I928" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J928" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K928" t="str">
+        <v/>
+      </c>
+      <c r="L928" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="str">
+        <v>C2026.0928</v>
+      </c>
+      <c r="B929" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C929" t="str">
+        <v>53490375</v>
+      </c>
+      <c r="D929" t="str">
+        <v>BARRA DE LIGAÇÃO SX</v>
+      </c>
+      <c r="E929" t="str">
+        <v>15</v>
+      </c>
+      <c r="F929" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G929" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H929" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I929" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J929" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K929" t="str">
+        <v/>
+      </c>
+      <c r="L929" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="str">
+        <v>C2026.0929</v>
+      </c>
+      <c r="B930" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C930" t="str">
+        <v>53490377</v>
+      </c>
+      <c r="D930" t="str">
+        <v>PEÇA DE LIGAÇÃO DX</v>
+      </c>
+      <c r="E930" t="str">
+        <v>15</v>
+      </c>
+      <c r="F930" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G930" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H930" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I930" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J930" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K930" t="str">
+        <v/>
+      </c>
+      <c r="L930" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="str">
+        <v>C2026.0930</v>
+      </c>
+      <c r="B931" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C931" t="str">
+        <v>53489671</v>
+      </c>
+      <c r="D931" t="str">
+        <v>CONJUNTO TRANSVERSAL TRASEIRO</v>
+      </c>
+      <c r="E931" t="str">
+        <v>15</v>
+      </c>
+      <c r="F931" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G931" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H931" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I931" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J931" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K931" t="str">
+        <v/>
+      </c>
+      <c r="L931" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="str">
+        <v>C2026.0931</v>
+      </c>
+      <c r="B932" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C932" t="str">
+        <v>53489671</v>
+      </c>
+      <c r="D932" t="str">
+        <v>CONJUNTO TRANSVERSAL TRASEIRO</v>
+      </c>
+      <c r="E932" t="str">
+        <v>15</v>
+      </c>
+      <c r="F932" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G932" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H932" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I932" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J932" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K932" t="str">
+        <v/>
+      </c>
+      <c r="L932" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="str">
+        <v>C2026.0932</v>
+      </c>
+      <c r="B933" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C933" t="str">
+        <v>53489671</v>
+      </c>
+      <c r="D933" t="str">
+        <v>CONJUNTO TRANSVERSAL TRASEIRO</v>
+      </c>
+      <c r="E933" t="str">
+        <v>15</v>
+      </c>
+      <c r="F933" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G933" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H933" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I933" t="str">
+        <v>CMM GLOBAL</v>
+      </c>
+      <c r="J933" t="str">
+        <v>GEOMETRIA</v>
+      </c>
+      <c r="K933" t="str">
+        <v/>
+      </c>
+      <c r="L933" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="str">
+        <v>C2026.0933</v>
+      </c>
+      <c r="B934" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C934" t="str">
+        <v>52213270</v>
+      </c>
+      <c r="D934" t="str">
+        <v>TORRESMO NEW LT</v>
+      </c>
+      <c r="E934">
+        <v>15</v>
+      </c>
+      <c r="F934" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G934" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H934" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I934" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J934" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K934" t="str">
+        <v/>
+      </c>
+      <c r="L934" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="str">
+        <v>C2026.0934</v>
+      </c>
+      <c r="B935" t="str">
+        <v>09/04/2026</v>
+      </c>
+      <c r="C935" t="str">
+        <v>52213270</v>
+      </c>
+      <c r="D935" t="str">
+        <v>TORRESMO NEW LT</v>
+      </c>
+      <c r="E935">
+        <v>15</v>
+      </c>
+      <c r="F935" t="str">
+        <v>QUALIDADE</v>
+      </c>
+      <c r="G935" t="str">
+        <v>luis</v>
+      </c>
+      <c r="H935" t="str">
+        <v>2º TURNO</v>
+      </c>
+      <c r="I935" t="str">
+        <v>METRASCAN</v>
+      </c>
+      <c r="J935" t="str">
+        <v>ANÁLISE DIMENSIONAL</v>
+      </c>
+      <c r="K935" t="str">
+        <v/>
+      </c>
+      <c r="L935" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L861"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L935"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>